<commit_message>
Actualizar datos de bicicleteros y agregar fotografías
</commit_message>
<xml_diff>
--- a/BICICLETERO 2026.xlsx
+++ b/BICICLETERO 2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Desktop\BICICLETERO\ConceptoStyle\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Concepto Style\Desktop\BICICLETERO 2.0\bicicletero\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A2EB1ED-FD91-47E0-B23D-F6CBF6FD4086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3FF9420-D6E1-488D-93B8-90DB8895628B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2325" yWindow="825" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="212">
   <si>
     <t>ESPACIO</t>
   </si>
@@ -593,6 +593,75 @@
   </si>
   <si>
     <t>se mudo</t>
+  </si>
+  <si>
+    <t>1.jpeg</t>
+  </si>
+  <si>
+    <t>2.jpeg</t>
+  </si>
+  <si>
+    <t>3.jpeg</t>
+  </si>
+  <si>
+    <t>4.jpeg</t>
+  </si>
+  <si>
+    <t>5.jpeg</t>
+  </si>
+  <si>
+    <t>6.jpeg</t>
+  </si>
+  <si>
+    <t>7.jpeg</t>
+  </si>
+  <si>
+    <t>8.jpeg</t>
+  </si>
+  <si>
+    <t>9.jpeg</t>
+  </si>
+  <si>
+    <t>10.jpeg</t>
+  </si>
+  <si>
+    <t>11.jpeg</t>
+  </si>
+  <si>
+    <t>12.jpeg</t>
+  </si>
+  <si>
+    <t>13.jpeg</t>
+  </si>
+  <si>
+    <t>14.jpeg</t>
+  </si>
+  <si>
+    <t>15.jpeg</t>
+  </si>
+  <si>
+    <t>16.jpeg</t>
+  </si>
+  <si>
+    <t>17.jpeg</t>
+  </si>
+  <si>
+    <t>18.jpeg</t>
+  </si>
+  <si>
+    <t>19.jpeg</t>
+  </si>
+  <si>
+    <t>20.jpeg</t>
+  </si>
+  <si>
+    <t>21.jpeg</t>
+  </si>
+  <si>
+    <t>23.jpeg</t>
+  </si>
+  <si>
+    <t>77.jpeg</t>
   </si>
 </sst>
 </file>
@@ -838,22 +907,6 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF6F8F9"/>
@@ -877,13 +930,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Hoja 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1118,7 +1187,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J83"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.28515625" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -1176,7 +1245,9 @@
       <c r="G2" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H2" s="5"/>
+      <c r="H2" s="6" t="s">
+        <v>189</v>
+      </c>
       <c r="I2" s="5"/>
       <c r="J2" s="5"/>
     </row>
@@ -1194,7 +1265,9 @@
       <c r="G3" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H3" s="5"/>
+      <c r="H3" s="6" t="s">
+        <v>190</v>
+      </c>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
     </row>
@@ -1212,7 +1285,9 @@
       <c r="G4" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H4" s="5"/>
+      <c r="H4" s="6" t="s">
+        <v>191</v>
+      </c>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
     </row>
@@ -1230,7 +1305,9 @@
       <c r="G5" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H5" s="5"/>
+      <c r="H5" s="6" t="s">
+        <v>192</v>
+      </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
     </row>
@@ -1248,7 +1325,9 @@
       <c r="G6" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H6" s="5"/>
+      <c r="H6" s="6" t="s">
+        <v>193</v>
+      </c>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
     </row>
@@ -1266,7 +1345,9 @@
       <c r="G7" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H7" s="5"/>
+      <c r="H7" s="6" t="s">
+        <v>194</v>
+      </c>
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
     </row>
@@ -1284,7 +1365,9 @@
       <c r="G8" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H8" s="5"/>
+      <c r="H8" s="6" t="s">
+        <v>195</v>
+      </c>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
     </row>
@@ -1302,7 +1385,9 @@
       <c r="G9" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H9" s="5"/>
+      <c r="H9" s="6" t="s">
+        <v>196</v>
+      </c>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
     </row>
@@ -1320,7 +1405,9 @@
       <c r="G10" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H10" s="5"/>
+      <c r="H10" s="6" t="s">
+        <v>197</v>
+      </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
     </row>
@@ -1338,7 +1425,9 @@
       <c r="G11" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H11" s="5"/>
+      <c r="H11" s="6" t="s">
+        <v>198</v>
+      </c>
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
     </row>
@@ -1356,7 +1445,9 @@
       <c r="G12" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H12" s="5"/>
+      <c r="H12" s="6" t="s">
+        <v>199</v>
+      </c>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
     </row>
@@ -1374,7 +1465,9 @@
       <c r="G13" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H13" s="5"/>
+      <c r="H13" s="6" t="s">
+        <v>200</v>
+      </c>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
     </row>
@@ -1392,7 +1485,9 @@
       <c r="G14" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H14" s="5"/>
+      <c r="H14" s="6" t="s">
+        <v>201</v>
+      </c>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
     </row>
@@ -1410,7 +1505,9 @@
       <c r="G15" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H15" s="5"/>
+      <c r="H15" s="6" t="s">
+        <v>202</v>
+      </c>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
     </row>
@@ -1428,7 +1525,9 @@
       <c r="G16" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H16" s="5"/>
+      <c r="H16" s="6" t="s">
+        <v>203</v>
+      </c>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
     </row>
@@ -1446,7 +1545,9 @@
       <c r="G17" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H17" s="5"/>
+      <c r="H17" s="6" t="s">
+        <v>204</v>
+      </c>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
     </row>
@@ -1464,7 +1565,9 @@
       <c r="G18" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H18" s="5"/>
+      <c r="H18" s="6" t="s">
+        <v>205</v>
+      </c>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
     </row>
@@ -1482,7 +1585,9 @@
       <c r="G19" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H19" s="5"/>
+      <c r="H19" s="6" t="s">
+        <v>206</v>
+      </c>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
     </row>
@@ -1500,7 +1605,9 @@
       <c r="G20" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H20" s="5"/>
+      <c r="H20" s="6" t="s">
+        <v>207</v>
+      </c>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
     </row>
@@ -1518,7 +1625,9 @@
       <c r="G21" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H21" s="5"/>
+      <c r="H21" s="6" t="s">
+        <v>208</v>
+      </c>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
     </row>
@@ -1536,7 +1645,9 @@
       <c r="G22" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H22" s="5"/>
+      <c r="H22" s="6" t="s">
+        <v>209</v>
+      </c>
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
     </row>
@@ -1578,7 +1689,9 @@
       <c r="G24" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="H24" s="5"/>
+      <c r="H24" s="6" t="s">
+        <v>210</v>
+      </c>
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
     </row>
@@ -3038,7 +3151,9 @@
       <c r="G79" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="H79" s="5"/>
+      <c r="H79" s="6" t="s">
+        <v>211</v>
+      </c>
       <c r="I79" s="5"/>
       <c r="J79" s="5"/>
     </row>
@@ -3156,7 +3271,7 @@
   <customSheetViews>
     <customSheetView guid="{77038CD4-2297-4E69-A928-9CF498AA6CA5}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:J83" xr:uid="{107E50ED-EB0B-4F62-A6F5-D7DE6CEE1B54}"/>
+      <autoFilter ref="A1:J83" xr:uid="{1C586E98-7F26-4B30-BA7A-136B29AF2F17}"/>
     </customSheetView>
   </customSheetViews>
   <dataValidations count="1">
@@ -3224,12 +3339,13 @@
     <hyperlink ref="H81" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
     <hyperlink ref="H82" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
     <hyperlink ref="H83" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="H2" r:id="rId60" display="22.jpeg" xr:uid="{CB170EA3-56E5-49B0-BE90-CB48DE40BD7E}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup fitToHeight="0" pageOrder="overThenDown" orientation="portrait" cellComments="atEnd"/>
   <tableParts count="1">
-    <tablePart r:id="rId60"/>
+    <tablePart r:id="rId61"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>